<commit_message>
Refactor: Refatorando alguns requisitos no backlog
</commit_message>
<xml_diff>
--- a/Documentações/Backlog.xlsx
+++ b/Documentações/Backlog.xlsx
@@ -5,19 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathe\OneDrive\Área de Trabalho\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\albuq\Repositorios\ThermoChain\Documentações\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BBD663-2B8F-404B-A035-3EA7C7743808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F99A68F-2191-4E2A-BE6E-76473101E5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88668B19-0EBA-47FC-AF05-5256D7A9BC46}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="120">
   <si>
     <t>Projeto no github</t>
   </si>
@@ -409,6 +406,18 @@
   </si>
   <si>
     <t>10/02/26 - 03/06/26</t>
+  </si>
+  <si>
+    <t>Dashboard intregado com o Bd</t>
+  </si>
+  <si>
+    <t>Desenvolver uma dashboard integrado ao Banco de Dados</t>
+  </si>
+  <si>
+    <t>Site de login com CRUD</t>
+  </si>
+  <si>
+    <t>Desenvolver um site de login sendo póssivel CRUD</t>
   </si>
 </sst>
 </file>
@@ -536,7 +545,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -596,11 +605,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -681,9 +703,48 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2423,15 +2484,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>599515</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>169208</xdr:rowOff>
+      <xdr:colOff>420222</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>158002</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>997323</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>11206</xdr:rowOff>
+      <xdr:colOff>818030</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2457,372 +2518,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Planilha1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="1">
-          <cell r="N1" t="str">
-            <v>Meta Ideal</v>
-          </cell>
-          <cell r="O1" t="str">
-            <v>Pendente</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="M2">
-            <v>0</v>
-          </cell>
-          <cell r="N2">
-            <v>360</v>
-          </cell>
-          <cell r="O2">
-            <v>370</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="M3">
-            <v>1</v>
-          </cell>
-          <cell r="N3">
-            <v>348</v>
-          </cell>
-          <cell r="O3">
-            <v>358</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="M4">
-            <v>2</v>
-          </cell>
-          <cell r="N4">
-            <v>336</v>
-          </cell>
-          <cell r="O4">
-            <v>346</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="M5">
-            <v>3</v>
-          </cell>
-          <cell r="N5">
-            <v>324</v>
-          </cell>
-          <cell r="O5">
-            <v>334</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="M6">
-            <v>4</v>
-          </cell>
-          <cell r="N6">
-            <v>312</v>
-          </cell>
-          <cell r="O6">
-            <v>322</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="M7">
-            <v>5</v>
-          </cell>
-          <cell r="N7">
-            <v>300</v>
-          </cell>
-          <cell r="O7">
-            <v>310</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="M8">
-            <v>6</v>
-          </cell>
-          <cell r="N8">
-            <v>288</v>
-          </cell>
-          <cell r="O8">
-            <v>298</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="M9">
-            <v>7</v>
-          </cell>
-          <cell r="N9">
-            <v>276</v>
-          </cell>
-          <cell r="O9">
-            <v>286</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="M10">
-            <v>8</v>
-          </cell>
-          <cell r="N10">
-            <v>264</v>
-          </cell>
-          <cell r="O10">
-            <v>274</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="M11">
-            <v>9</v>
-          </cell>
-          <cell r="N11">
-            <v>252</v>
-          </cell>
-          <cell r="O11">
-            <v>262</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="M12">
-            <v>10</v>
-          </cell>
-          <cell r="N12">
-            <v>240</v>
-          </cell>
-          <cell r="O12">
-            <v>240</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="M13">
-            <v>11</v>
-          </cell>
-          <cell r="N13">
-            <v>228</v>
-          </cell>
-          <cell r="O13">
-            <v>228</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="M14">
-            <v>12</v>
-          </cell>
-          <cell r="N14">
-            <v>216</v>
-          </cell>
-          <cell r="O14">
-            <v>216</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="M15">
-            <v>13</v>
-          </cell>
-          <cell r="N15">
-            <v>204</v>
-          </cell>
-          <cell r="O15">
-            <v>204</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="M16">
-            <v>14</v>
-          </cell>
-          <cell r="N16">
-            <v>192</v>
-          </cell>
-          <cell r="O16">
-            <v>192</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="M17">
-            <v>15</v>
-          </cell>
-          <cell r="N17">
-            <v>180</v>
-          </cell>
-          <cell r="O17">
-            <v>180</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="M18">
-            <v>16</v>
-          </cell>
-          <cell r="N18">
-            <v>168</v>
-          </cell>
-          <cell r="O18">
-            <v>168</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="M19">
-            <v>17</v>
-          </cell>
-          <cell r="N19">
-            <v>156</v>
-          </cell>
-          <cell r="O19">
-            <v>156</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="M20">
-            <v>18</v>
-          </cell>
-          <cell r="N20">
-            <v>144</v>
-          </cell>
-          <cell r="O20">
-            <v>144</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="M21">
-            <v>19</v>
-          </cell>
-          <cell r="N21">
-            <v>132</v>
-          </cell>
-          <cell r="O21">
-            <v>132</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="M22">
-            <v>20</v>
-          </cell>
-          <cell r="N22">
-            <v>120</v>
-          </cell>
-          <cell r="O22">
-            <v>120</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="M23">
-            <v>21</v>
-          </cell>
-          <cell r="N23">
-            <v>108</v>
-          </cell>
-          <cell r="O23">
-            <v>98</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="M24">
-            <v>22</v>
-          </cell>
-          <cell r="N24">
-            <v>96</v>
-          </cell>
-          <cell r="O24">
-            <v>86</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="M25">
-            <v>23</v>
-          </cell>
-          <cell r="N25">
-            <v>84</v>
-          </cell>
-          <cell r="O25">
-            <v>74</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="M26">
-            <v>24</v>
-          </cell>
-          <cell r="N26">
-            <v>72</v>
-          </cell>
-          <cell r="O26">
-            <v>62</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="M27">
-            <v>25</v>
-          </cell>
-          <cell r="N27">
-            <v>60</v>
-          </cell>
-          <cell r="O27">
-            <v>50</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="M28">
-            <v>26</v>
-          </cell>
-          <cell r="N28">
-            <v>48</v>
-          </cell>
-          <cell r="O28">
-            <v>38</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="M29">
-            <v>27</v>
-          </cell>
-          <cell r="N29">
-            <v>36</v>
-          </cell>
-          <cell r="O29">
-            <v>26</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="M30">
-            <v>28</v>
-          </cell>
-          <cell r="N30">
-            <v>24</v>
-          </cell>
-          <cell r="O30">
-            <v>14</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="M31">
-            <v>29</v>
-          </cell>
-          <cell r="N31">
-            <v>12</v>
-          </cell>
-          <cell r="O31">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="M32">
-            <v>30</v>
-          </cell>
-          <cell r="N32">
-            <v>0</v>
-          </cell>
-          <cell r="O32">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4991,28 +4686,28 @@
       </c>
     </row>
     <row r="39" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E39" s="19" t="s">
+      <c r="E39" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="F39" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="G39" s="20" t="s">
+      <c r="G39" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="H39" s="25" t="s">
+      <c r="H39" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="I39" s="25">
+      <c r="I39" s="35">
         <v>8</v>
       </c>
-      <c r="J39" s="22">
+      <c r="J39" s="36">
         <v>2</v>
       </c>
-      <c r="K39" s="28" t="s">
+      <c r="K39" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="L39" s="4"/>
+      <c r="L39" s="38"/>
       <c r="N39" s="6">
         <v>36</v>
       </c>
@@ -5037,6 +4732,28 @@
       </c>
     </row>
     <row r="40" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="E40" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="F40" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="G40" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H40" s="41" t="s">
+        <v>64</v>
+      </c>
+      <c r="I40" s="41">
+        <v>21</v>
+      </c>
+      <c r="J40" s="12">
+        <v>1</v>
+      </c>
+      <c r="K40" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="L40" s="39"/>
       <c r="N40" s="6">
         <v>37</v>
       </c>
@@ -5061,6 +4778,28 @@
       </c>
     </row>
     <row r="41" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="E41" s="42" t="s">
+        <v>118</v>
+      </c>
+      <c r="F41" s="42" t="s">
+        <v>119</v>
+      </c>
+      <c r="G41" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="H41" s="44" t="s">
+        <v>61</v>
+      </c>
+      <c r="I41" s="44">
+        <v>13</v>
+      </c>
+      <c r="J41" s="45">
+        <v>2</v>
+      </c>
+      <c r="K41" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="L41" s="42"/>
       <c r="N41" s="6">
         <v>38</v>
       </c>
@@ -5157,6 +4896,7 @@
       </c>
     </row>
     <row r="45" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="G45" s="47"/>
       <c r="N45" s="6">
         <v>42</v>
       </c>
@@ -5713,7 +5453,7 @@
         <v>3</v>
       </c>
       <c r="P69" s="6">
-        <f t="shared" ref="P69:P117" si="6">P68-$O$4</f>
+        <f t="shared" ref="P69:P93" si="6">P68-$O$4</f>
         <v>74</v>
       </c>
       <c r="Q69" s="6"/>
@@ -6764,14 +6504,6 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="N3:N117">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6780,6 +6512,14 @@
         <color rgb="FF63BE7B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat: Backlog e home atualizados
</commit_message>
<xml_diff>
--- a/Documentações/Backlog.xlsx
+++ b/Documentações/Backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\albuq\Repositorios\ThermoChain\Documentações\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathe\OneDrive\Área de Trabalho\ThermoChain\Documentações\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F99A68F-2191-4E2A-BE6E-76473101E5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9043B5DC-6179-4972-B9FC-F6B2F63B3114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88668B19-0EBA-47FC-AF05-5256D7A9BC46}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{88668B19-0EBA-47FC-AF05-5256D7A9BC46}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -622,7 +622,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -731,20 +731,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1253,10 +1245,10 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Planilha1!$R$3:$R$117</c:f>
+              <c:f>Planilha1!$R$3:$R$58</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="115"/>
+                <c:ptCount val="56"/>
                 <c:pt idx="0">
                   <c:v>272</c:v>
                 </c:pt>
@@ -1423,184 +1415,7 @@
                   <c:v>103</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="78">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="79">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="80">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="81">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="82">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="83">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="84">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="85">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="86">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="87">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="88">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="89">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="90">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="91">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="92">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="93">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="94">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="95">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="96">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="97">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="98">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="99">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="100">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="101">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="102">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="103">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="104">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="105">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="106">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="107">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="108">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="109">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="110">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="111">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="112">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="113">
-                  <c:v>103</c:v>
-                </c:pt>
-                <c:pt idx="114">
-                  <c:v>103</c:v>
+                  <c:v>90</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2838,29 +2653,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{552007D4-E79E-4A61-AC31-FF3BEBBC1490}">
   <dimension ref="A2:T118"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.5703125" customWidth="1"/>
+    <col min="1" max="1" width="28.5546875" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="5" max="5" width="45.7109375" customWidth="1"/>
-    <col min="6" max="6" width="53.28515625" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" customWidth="1"/>
-    <col min="11" max="11" width="12.7109375" customWidth="1"/>
-    <col min="12" max="12" width="15.140625" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" customWidth="1"/>
-    <col min="16" max="16" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="45.6640625" customWidth="1"/>
+    <col min="6" max="6" width="53.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="9.6640625" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
+    <col min="11" max="11" width="12.6640625" customWidth="1"/>
+    <col min="12" max="12" width="15.109375" customWidth="1"/>
+    <col min="13" max="13" width="8.88671875" customWidth="1"/>
+    <col min="14" max="14" width="10.6640625" customWidth="1"/>
+    <col min="15" max="15" width="12.6640625" customWidth="1"/>
+    <col min="16" max="16" width="17.6640625" customWidth="1"/>
     <col min="17" max="17" width="21" customWidth="1"/>
-    <col min="18" max="18" width="13.5703125" customWidth="1"/>
-    <col min="19" max="19" width="13.85546875" customWidth="1"/>
-    <col min="20" max="20" width="11.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13.5546875" customWidth="1"/>
+    <col min="19" max="19" width="13.88671875" customWidth="1"/>
+    <col min="20" max="20" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
         <v>59</v>
       </c>
@@ -2913,7 +2728,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="24" t="s">
         <v>63</v>
       </c>
@@ -2968,7 +2783,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
         <v>60</v>
       </c>
@@ -3026,7 +2841,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="27" t="s">
         <v>61</v>
       </c>
@@ -3083,7 +2898,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="26" t="s">
         <v>64</v>
       </c>
@@ -3137,7 +2952,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="E7" s="19" t="s">
         <v>4</v>
       </c>
@@ -3185,7 +3000,7 @@
         <v>46067</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>101</v>
       </c>
@@ -3240,7 +3055,7 @@
         <v>46068</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>102</v>
       </c>
@@ -3294,7 +3109,7 @@
         <v>46069</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>103</v>
       </c>
@@ -3349,7 +3164,7 @@
         <v>46070</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="30" t="s">
         <v>114</v>
       </c>
@@ -3403,7 +3218,7 @@
         <v>46071</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="E12" s="19" t="s">
         <v>9</v>
       </c>
@@ -3451,7 +3266,7 @@
         <v>46072</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="E13" s="19" t="s">
         <v>10</v>
@@ -3500,7 +3315,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="E14" s="19" t="s">
         <v>11</v>
@@ -3549,7 +3364,7 @@
         <v>46074</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="E15" s="19" t="s">
         <v>12</v>
       </c>
@@ -3597,7 +3412,7 @@
         <v>46075</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="E16" s="19" t="s">
         <v>13</v>
       </c>
@@ -3645,7 +3460,7 @@
         <v>46076</v>
       </c>
     </row>
-    <row r="17" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E17" s="19" t="s">
         <v>14</v>
       </c>
@@ -3693,7 +3508,7 @@
         <v>46077</v>
       </c>
     </row>
-    <row r="18" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E18" s="19" t="s">
         <v>15</v>
       </c>
@@ -3741,7 +3556,7 @@
         <v>46078</v>
       </c>
     </row>
-    <row r="19" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E19" s="19" t="s">
         <v>24</v>
       </c>
@@ -3789,7 +3604,7 @@
         <v>46079</v>
       </c>
     </row>
-    <row r="20" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E20" s="19" t="s">
         <v>25</v>
       </c>
@@ -3835,7 +3650,7 @@
         <v>46080</v>
       </c>
     </row>
-    <row r="21" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E21" s="19" t="s">
         <v>26</v>
       </c>
@@ -3883,11 +3698,11 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="22" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="17" t="s">
         <v>76</v>
       </c>
       <c r="G22" s="20" t="s">
@@ -3931,7 +3746,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="23" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E23" s="19" t="s">
         <v>28</v>
       </c>
@@ -3979,7 +3794,7 @@
         <v>46083</v>
       </c>
     </row>
-    <row r="24" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E24" s="19" t="s">
         <v>29</v>
       </c>
@@ -4027,7 +3842,7 @@
         <v>46084</v>
       </c>
     </row>
-    <row r="25" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E25" s="19" t="s">
         <v>30</v>
       </c>
@@ -4073,7 +3888,7 @@
         <v>46085</v>
       </c>
     </row>
-    <row r="26" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E26" s="19" t="s">
         <v>31</v>
       </c>
@@ -4121,7 +3936,7 @@
         <v>46086</v>
       </c>
     </row>
-    <row r="27" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E27" s="19" t="s">
         <v>32</v>
       </c>
@@ -4169,7 +3984,7 @@
         <v>46087</v>
       </c>
     </row>
-    <row r="28" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E28" s="19" t="s">
         <v>33</v>
       </c>
@@ -4217,7 +4032,7 @@
         <v>46088</v>
       </c>
     </row>
-    <row r="29" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E29" s="19" t="s">
         <v>34</v>
       </c>
@@ -4265,7 +4080,7 @@
         <v>46089</v>
       </c>
     </row>
-    <row r="30" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E30" s="19" t="s">
         <v>35</v>
       </c>
@@ -4313,7 +4128,7 @@
         <v>46090</v>
       </c>
     </row>
-    <row r="31" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E31" s="19" t="s">
         <v>36</v>
       </c>
@@ -4359,7 +4174,7 @@
         <v>46091</v>
       </c>
     </row>
-    <row r="32" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E32" s="19" t="s">
         <v>37</v>
       </c>
@@ -4407,7 +4222,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="33" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E33" s="19" t="s">
         <v>38</v>
       </c>
@@ -4455,7 +4270,7 @@
         <v>46093</v>
       </c>
     </row>
-    <row r="34" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E34" s="19" t="s">
         <v>39</v>
       </c>
@@ -4501,7 +4316,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="35" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E35" s="19" t="s">
         <v>90</v>
       </c>
@@ -4547,7 +4362,7 @@
         <v>46095</v>
       </c>
     </row>
-    <row r="36" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E36" s="19" t="s">
         <v>91</v>
       </c>
@@ -4593,7 +4408,7 @@
         <v>46096</v>
       </c>
     </row>
-    <row r="37" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E37" s="19" t="s">
         <v>92</v>
       </c>
@@ -4639,7 +4454,7 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="38" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E38" s="19" t="s">
         <v>93</v>
       </c>
@@ -4685,7 +4500,7 @@
         <v>46098</v>
       </c>
     </row>
-    <row r="39" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E39" s="31" t="s">
         <v>94</v>
       </c>
@@ -4731,7 +4546,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="40" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="5:19" x14ac:dyDescent="0.3">
       <c r="E40" s="32" t="s">
         <v>116</v>
       </c>
@@ -4777,29 +4592,29 @@
         <v>46100</v>
       </c>
     </row>
-    <row r="41" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="E41" s="42" t="s">
+    <row r="41" spans="5:19" x14ac:dyDescent="0.3">
+      <c r="E41" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="F41" s="42" t="s">
+      <c r="F41" s="39" t="s">
         <v>119</v>
       </c>
-      <c r="G41" s="43" t="s">
+      <c r="G41" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="H41" s="44" t="s">
+      <c r="H41" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="I41" s="44">
+      <c r="I41" s="42">
         <v>13</v>
       </c>
-      <c r="J41" s="45">
+      <c r="J41" s="43">
         <v>2</v>
       </c>
-      <c r="K41" s="46" t="s">
+      <c r="K41" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="L41" s="42"/>
+      <c r="L41" s="39"/>
       <c r="N41" s="6">
         <v>38</v>
       </c>
@@ -4823,7 +4638,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="42" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="5:19" x14ac:dyDescent="0.3">
       <c r="N42" s="6">
         <v>39</v>
       </c>
@@ -4847,7 +4662,7 @@
         <v>46102</v>
       </c>
     </row>
-    <row r="43" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="5:19" x14ac:dyDescent="0.3">
       <c r="N43" s="6">
         <v>40</v>
       </c>
@@ -4871,7 +4686,7 @@
         <v>46103</v>
       </c>
     </row>
-    <row r="44" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="5:19" x14ac:dyDescent="0.3">
       <c r="N44" s="6">
         <v>41</v>
       </c>
@@ -4895,8 +4710,7 @@
         <v>46104</v>
       </c>
     </row>
-    <row r="45" spans="5:19" x14ac:dyDescent="0.25">
-      <c r="G45" s="47"/>
+    <row r="45" spans="5:19" x14ac:dyDescent="0.3">
       <c r="N45" s="6">
         <v>42</v>
       </c>
@@ -4920,7 +4734,7 @@
         <v>46105</v>
       </c>
     </row>
-    <row r="46" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="5:19" x14ac:dyDescent="0.3">
       <c r="N46" s="6">
         <v>43</v>
       </c>
@@ -4944,7 +4758,7 @@
         <v>46106</v>
       </c>
     </row>
-    <row r="47" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="5:19" x14ac:dyDescent="0.3">
       <c r="N47" s="6">
         <v>44</v>
       </c>
@@ -4968,7 +4782,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="48" spans="5:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="5:19" x14ac:dyDescent="0.3">
       <c r="N48" s="6">
         <v>45</v>
       </c>
@@ -4992,7 +4806,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="49" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="49" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N49" s="6">
         <v>46</v>
       </c>
@@ -5016,7 +4830,7 @@
         <v>46109</v>
       </c>
     </row>
-    <row r="50" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N50" s="6">
         <v>47</v>
       </c>
@@ -5040,7 +4854,7 @@
         <v>46110</v>
       </c>
     </row>
-    <row r="51" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N51" s="6">
         <v>48</v>
       </c>
@@ -5064,7 +4878,7 @@
         <v>46111</v>
       </c>
     </row>
-    <row r="52" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N52" s="6">
         <v>49</v>
       </c>
@@ -5088,7 +4902,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="53" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="53" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N53" s="6">
         <v>50</v>
       </c>
@@ -5112,7 +4926,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="54" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N54" s="6">
         <v>51</v>
       </c>
@@ -5136,7 +4950,7 @@
         <v>46114</v>
       </c>
     </row>
-    <row r="55" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="55" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N55" s="6">
         <v>52</v>
       </c>
@@ -5148,7 +4962,9 @@
         <f t="shared" si="1"/>
         <v>116</v>
       </c>
-      <c r="Q55" s="6"/>
+      <c r="Q55" s="6">
+        <v>0</v>
+      </c>
       <c r="R55" s="6">
         <f t="shared" si="3"/>
         <v>103</v>
@@ -5158,7 +4974,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="56" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N56" s="6">
         <v>53</v>
       </c>
@@ -5170,7 +4986,9 @@
         <f t="shared" si="1"/>
         <v>113</v>
       </c>
-      <c r="Q56" s="6"/>
+      <c r="Q56" s="6">
+        <v>0</v>
+      </c>
       <c r="R56" s="6">
         <f t="shared" si="3"/>
         <v>103</v>
@@ -5180,7 +4998,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="57" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N57" s="6">
         <v>54</v>
       </c>
@@ -5192,7 +5010,9 @@
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="Q57" s="6"/>
+      <c r="Q57" s="6">
+        <v>0</v>
+      </c>
       <c r="R57" s="6">
         <f t="shared" si="3"/>
         <v>103</v>
@@ -5202,7 +5022,7 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="58" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N58" s="6">
         <v>55</v>
       </c>
@@ -5214,17 +5034,19 @@
         <f t="shared" si="1"/>
         <v>107</v>
       </c>
-      <c r="Q58" s="6"/>
+      <c r="Q58" s="6">
+        <v>13</v>
+      </c>
       <c r="R58" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S58" s="15">
         <f t="shared" si="2"/>
         <v>46118</v>
       </c>
     </row>
-    <row r="59" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N59" s="6">
         <v>56</v>
       </c>
@@ -5239,14 +5061,14 @@
       <c r="Q59" s="6"/>
       <c r="R59" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S59" s="15">
         <f t="shared" si="2"/>
         <v>46119</v>
       </c>
     </row>
-    <row r="60" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N60" s="6">
         <v>57</v>
       </c>
@@ -5261,14 +5083,14 @@
       <c r="Q60" s="6"/>
       <c r="R60" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S60" s="15">
         <f t="shared" si="2"/>
         <v>46120</v>
       </c>
     </row>
-    <row r="61" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="61" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N61" s="6">
         <v>58</v>
       </c>
@@ -5283,14 +5105,14 @@
       <c r="Q61" s="6"/>
       <c r="R61" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S61" s="15">
         <f t="shared" si="2"/>
         <v>46121</v>
       </c>
     </row>
-    <row r="62" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="62" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N62" s="6">
         <v>59</v>
       </c>
@@ -5305,14 +5127,14 @@
       <c r="Q62" s="6"/>
       <c r="R62" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S62" s="15">
         <f t="shared" si="2"/>
         <v>46122</v>
       </c>
     </row>
-    <row r="63" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="63" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N63" s="6">
         <v>60</v>
       </c>
@@ -5327,14 +5149,14 @@
       <c r="Q63" s="6"/>
       <c r="R63" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S63" s="15">
         <f t="shared" si="2"/>
         <v>46123</v>
       </c>
     </row>
-    <row r="64" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="64" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N64" s="6">
         <v>61</v>
       </c>
@@ -5349,14 +5171,14 @@
       <c r="Q64" s="6"/>
       <c r="R64" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S64" s="15">
         <f t="shared" si="2"/>
         <v>46124</v>
       </c>
     </row>
-    <row r="65" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N65" s="6">
         <v>62</v>
       </c>
@@ -5371,14 +5193,14 @@
       <c r="Q65" s="6"/>
       <c r="R65" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S65" s="15">
         <f t="shared" si="2"/>
         <v>46125</v>
       </c>
     </row>
-    <row r="66" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N66" s="6">
         <v>63</v>
       </c>
@@ -5393,14 +5215,14 @@
       <c r="Q66" s="6"/>
       <c r="R66" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S66" s="15">
         <f t="shared" si="2"/>
         <v>46126</v>
       </c>
     </row>
-    <row r="67" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N67" s="6">
         <v>64</v>
       </c>
@@ -5415,14 +5237,14 @@
       <c r="Q67" s="6"/>
       <c r="R67" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S67" s="15">
         <f t="shared" si="2"/>
         <v>46127</v>
       </c>
     </row>
-    <row r="68" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N68" s="6">
         <v>65</v>
       </c>
@@ -5437,14 +5259,14 @@
       <c r="Q68" s="6"/>
       <c r="R68" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S68" s="15">
         <f t="shared" si="2"/>
         <v>46128</v>
       </c>
     </row>
-    <row r="69" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N69" s="6">
         <v>66</v>
       </c>
@@ -5459,14 +5281,14 @@
       <c r="Q69" s="6"/>
       <c r="R69" s="6">
         <f t="shared" si="3"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S69" s="15">
         <f t="shared" ref="S69:S117" si="7">S68+1</f>
         <v>46129</v>
       </c>
     </row>
-    <row r="70" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N70" s="6">
         <v>67</v>
       </c>
@@ -5481,14 +5303,14 @@
       <c r="Q70" s="6"/>
       <c r="R70" s="6">
         <f t="shared" ref="R70:R117" si="8">IF(Q70&lt;&gt;"",R69-Q70,R69)</f>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S70" s="15">
         <f t="shared" si="7"/>
         <v>46130</v>
       </c>
     </row>
-    <row r="71" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N71" s="6">
         <v>68</v>
       </c>
@@ -5503,14 +5325,14 @@
       <c r="Q71" s="6"/>
       <c r="R71" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S71" s="15">
         <f t="shared" si="7"/>
         <v>46131</v>
       </c>
     </row>
-    <row r="72" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N72" s="6">
         <v>69</v>
       </c>
@@ -5525,14 +5347,14 @@
       <c r="Q72" s="6"/>
       <c r="R72" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S72" s="15">
         <f t="shared" si="7"/>
         <v>46132</v>
       </c>
     </row>
-    <row r="73" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N73" s="6">
         <v>70</v>
       </c>
@@ -5547,14 +5369,14 @@
       <c r="Q73" s="6"/>
       <c r="R73" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S73" s="15">
         <f t="shared" si="7"/>
         <v>46133</v>
       </c>
     </row>
-    <row r="74" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N74" s="6">
         <v>71</v>
       </c>
@@ -5569,14 +5391,14 @@
       <c r="Q74" s="6"/>
       <c r="R74" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S74" s="15">
         <f t="shared" si="7"/>
         <v>46134</v>
       </c>
     </row>
-    <row r="75" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N75" s="6">
         <v>72</v>
       </c>
@@ -5591,14 +5413,14 @@
       <c r="Q75" s="6"/>
       <c r="R75" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S75" s="16">
         <f t="shared" si="7"/>
         <v>46135</v>
       </c>
     </row>
-    <row r="76" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N76" s="6">
         <v>73</v>
       </c>
@@ -5613,14 +5435,14 @@
       <c r="Q76" s="6"/>
       <c r="R76" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S76" s="16">
         <f t="shared" si="7"/>
         <v>46136</v>
       </c>
     </row>
-    <row r="77" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="77" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N77" s="6">
         <v>74</v>
       </c>
@@ -5635,14 +5457,14 @@
       <c r="Q77" s="6"/>
       <c r="R77" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S77" s="16">
         <f t="shared" si="7"/>
         <v>46137</v>
       </c>
     </row>
-    <row r="78" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="78" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N78" s="6">
         <v>75</v>
       </c>
@@ -5657,14 +5479,14 @@
       <c r="Q78" s="6"/>
       <c r="R78" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S78" s="16">
         <f t="shared" si="7"/>
         <v>46138</v>
       </c>
     </row>
-    <row r="79" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="79" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N79" s="6">
         <v>76</v>
       </c>
@@ -5679,14 +5501,14 @@
       <c r="Q79" s="6"/>
       <c r="R79" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S79" s="16">
         <f t="shared" si="7"/>
         <v>46139</v>
       </c>
     </row>
-    <row r="80" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="80" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N80" s="6">
         <v>77</v>
       </c>
@@ -5701,14 +5523,14 @@
       <c r="Q80" s="6"/>
       <c r="R80" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S80" s="16">
         <f t="shared" si="7"/>
         <v>46140</v>
       </c>
     </row>
-    <row r="81" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N81" s="6">
         <v>78</v>
       </c>
@@ -5723,14 +5545,14 @@
       <c r="Q81" s="6"/>
       <c r="R81" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S81" s="16">
         <f t="shared" si="7"/>
         <v>46141</v>
       </c>
     </row>
-    <row r="82" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N82" s="6">
         <v>79</v>
       </c>
@@ -5745,14 +5567,14 @@
       <c r="Q82" s="6"/>
       <c r="R82" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S82" s="16">
         <f t="shared" si="7"/>
         <v>46142</v>
       </c>
     </row>
-    <row r="83" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="83" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N83" s="6">
         <v>80</v>
       </c>
@@ -5767,14 +5589,14 @@
       <c r="Q83" s="6"/>
       <c r="R83" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S83" s="16">
         <f t="shared" si="7"/>
         <v>46143</v>
       </c>
     </row>
-    <row r="84" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N84" s="6">
         <v>81</v>
       </c>
@@ -5789,14 +5611,14 @@
       <c r="Q84" s="6"/>
       <c r="R84" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S84" s="16">
         <f t="shared" si="7"/>
         <v>46144</v>
       </c>
     </row>
-    <row r="85" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N85" s="6">
         <v>82</v>
       </c>
@@ -5811,14 +5633,14 @@
       <c r="Q85" s="6"/>
       <c r="R85" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S85" s="16">
         <f t="shared" si="7"/>
         <v>46145</v>
       </c>
     </row>
-    <row r="86" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N86" s="6">
         <v>83</v>
       </c>
@@ -5833,14 +5655,14 @@
       <c r="Q86" s="6"/>
       <c r="R86" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S86" s="16">
         <f t="shared" si="7"/>
         <v>46146</v>
       </c>
     </row>
-    <row r="87" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N87" s="6">
         <v>84</v>
       </c>
@@ -5855,14 +5677,14 @@
       <c r="Q87" s="6"/>
       <c r="R87" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S87" s="16">
         <f t="shared" si="7"/>
         <v>46147</v>
       </c>
     </row>
-    <row r="88" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="88" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N88" s="6">
         <v>85</v>
       </c>
@@ -5877,14 +5699,14 @@
       <c r="Q88" s="6"/>
       <c r="R88" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S88" s="16">
         <f t="shared" si="7"/>
         <v>46148</v>
       </c>
     </row>
-    <row r="89" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="89" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N89" s="6">
         <v>86</v>
       </c>
@@ -5899,14 +5721,14 @@
       <c r="Q89" s="6"/>
       <c r="R89" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S89" s="16">
         <f t="shared" si="7"/>
         <v>46149</v>
       </c>
     </row>
-    <row r="90" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="90" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N90" s="6">
         <v>87</v>
       </c>
@@ -5921,14 +5743,14 @@
       <c r="Q90" s="6"/>
       <c r="R90" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S90" s="16">
         <f t="shared" si="7"/>
         <v>46150</v>
       </c>
     </row>
-    <row r="91" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="91" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N91" s="6">
         <v>88</v>
       </c>
@@ -5943,14 +5765,14 @@
       <c r="Q91" s="6"/>
       <c r="R91" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S91" s="16">
         <f t="shared" si="7"/>
         <v>46151</v>
       </c>
     </row>
-    <row r="92" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="92" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N92" s="6">
         <v>89</v>
       </c>
@@ -5965,14 +5787,14 @@
       <c r="Q92" s="6"/>
       <c r="R92" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S92" s="16">
         <f t="shared" si="7"/>
         <v>46152</v>
       </c>
     </row>
-    <row r="93" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="93" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N93" s="6">
         <v>90</v>
       </c>
@@ -5987,14 +5809,14 @@
       <c r="Q93" s="6"/>
       <c r="R93" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S93" s="16">
         <f t="shared" si="7"/>
         <v>46153</v>
       </c>
     </row>
-    <row r="94" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="94" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N94" s="6">
         <v>91</v>
       </c>
@@ -6008,14 +5830,14 @@
       <c r="Q94" s="6"/>
       <c r="R94" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S94" s="16">
         <f t="shared" si="7"/>
         <v>46154</v>
       </c>
     </row>
-    <row r="95" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="95" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N95" s="6">
         <v>92</v>
       </c>
@@ -6029,14 +5851,14 @@
       <c r="Q95" s="6"/>
       <c r="R95" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S95" s="16">
         <f t="shared" si="7"/>
         <v>46155</v>
       </c>
     </row>
-    <row r="96" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="96" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N96" s="6">
         <v>93</v>
       </c>
@@ -6050,14 +5872,14 @@
       <c r="Q96" s="6"/>
       <c r="R96" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S96" s="16">
         <f t="shared" si="7"/>
         <v>46156</v>
       </c>
     </row>
-    <row r="97" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="97" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N97" s="6">
         <v>94</v>
       </c>
@@ -6071,14 +5893,14 @@
       <c r="Q97" s="6"/>
       <c r="R97" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S97" s="16">
         <f t="shared" si="7"/>
         <v>46157</v>
       </c>
     </row>
-    <row r="98" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="98" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N98" s="6">
         <v>95</v>
       </c>
@@ -6092,14 +5914,14 @@
       <c r="Q98" s="6"/>
       <c r="R98" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S98" s="16">
         <f t="shared" si="7"/>
         <v>46158</v>
       </c>
     </row>
-    <row r="99" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="99" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N99" s="6">
         <v>96</v>
       </c>
@@ -6113,14 +5935,14 @@
       <c r="Q99" s="6"/>
       <c r="R99" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S99" s="16">
         <f t="shared" si="7"/>
         <v>46159</v>
       </c>
     </row>
-    <row r="100" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="100" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N100" s="6">
         <v>97</v>
       </c>
@@ -6134,14 +5956,14 @@
       <c r="Q100" s="6"/>
       <c r="R100" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S100" s="16">
         <f t="shared" si="7"/>
         <v>46160</v>
       </c>
     </row>
-    <row r="101" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="101" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N101" s="6">
         <v>98</v>
       </c>
@@ -6155,14 +5977,14 @@
       <c r="Q101" s="6"/>
       <c r="R101" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S101" s="16">
         <f t="shared" si="7"/>
         <v>46161</v>
       </c>
     </row>
-    <row r="102" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="102" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N102" s="6">
         <v>99</v>
       </c>
@@ -6176,14 +5998,14 @@
       <c r="Q102" s="6"/>
       <c r="R102" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S102" s="16">
         <f t="shared" si="7"/>
         <v>46162</v>
       </c>
     </row>
-    <row r="103" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="103" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N103" s="6">
         <v>100</v>
       </c>
@@ -6197,14 +6019,14 @@
       <c r="Q103" s="6"/>
       <c r="R103" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S103" s="16">
         <f t="shared" si="7"/>
         <v>46163</v>
       </c>
     </row>
-    <row r="104" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="104" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N104" s="6">
         <v>101</v>
       </c>
@@ -6218,14 +6040,14 @@
       <c r="Q104" s="6"/>
       <c r="R104" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S104" s="16">
         <f t="shared" si="7"/>
         <v>46164</v>
       </c>
     </row>
-    <row r="105" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="105" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N105" s="6">
         <v>102</v>
       </c>
@@ -6239,14 +6061,14 @@
       <c r="Q105" s="6"/>
       <c r="R105" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S105" s="16">
         <f t="shared" si="7"/>
         <v>46165</v>
       </c>
     </row>
-    <row r="106" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="106" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N106" s="6">
         <v>103</v>
       </c>
@@ -6260,14 +6082,14 @@
       <c r="Q106" s="6"/>
       <c r="R106" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S106" s="16">
         <f t="shared" si="7"/>
         <v>46166</v>
       </c>
     </row>
-    <row r="107" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="107" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N107" s="6">
         <v>104</v>
       </c>
@@ -6281,14 +6103,14 @@
       <c r="Q107" s="6"/>
       <c r="R107" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S107" s="16">
         <f t="shared" si="7"/>
         <v>46167</v>
       </c>
     </row>
-    <row r="108" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="108" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N108" s="6">
         <v>105</v>
       </c>
@@ -6302,14 +6124,14 @@
       <c r="Q108" s="6"/>
       <c r="R108" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S108" s="16">
         <f t="shared" si="7"/>
         <v>46168</v>
       </c>
     </row>
-    <row r="109" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="109" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N109" s="6">
         <v>106</v>
       </c>
@@ -6323,14 +6145,14 @@
       <c r="Q109" s="6"/>
       <c r="R109" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S109" s="16">
         <f t="shared" si="7"/>
         <v>46169</v>
       </c>
     </row>
-    <row r="110" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="110" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N110" s="6">
         <v>107</v>
       </c>
@@ -6344,14 +6166,14 @@
       <c r="Q110" s="6"/>
       <c r="R110" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S110" s="16">
         <f t="shared" si="7"/>
         <v>46170</v>
       </c>
     </row>
-    <row r="111" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="111" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N111" s="6">
         <v>108</v>
       </c>
@@ -6365,14 +6187,14 @@
       <c r="Q111" s="6"/>
       <c r="R111" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S111" s="16">
         <f t="shared" si="7"/>
         <v>46171</v>
       </c>
     </row>
-    <row r="112" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="112" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N112" s="6">
         <v>109</v>
       </c>
@@ -6386,14 +6208,14 @@
       <c r="Q112" s="6"/>
       <c r="R112" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S112" s="16">
         <f t="shared" si="7"/>
         <v>46172</v>
       </c>
     </row>
-    <row r="113" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="113" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N113" s="6">
         <v>110</v>
       </c>
@@ -6407,14 +6229,14 @@
       <c r="Q113" s="6"/>
       <c r="R113" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S113" s="16">
         <f t="shared" si="7"/>
         <v>46173</v>
       </c>
     </row>
-    <row r="114" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="114" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N114" s="6">
         <v>111</v>
       </c>
@@ -6428,14 +6250,14 @@
       <c r="Q114" s="6"/>
       <c r="R114" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S114" s="16">
         <f t="shared" si="7"/>
         <v>46174</v>
       </c>
     </row>
-    <row r="115" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="115" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N115" s="6">
         <v>112</v>
       </c>
@@ -6449,14 +6271,14 @@
       <c r="Q115" s="6"/>
       <c r="R115" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S115" s="16">
         <f t="shared" si="7"/>
         <v>46175</v>
       </c>
     </row>
-    <row r="116" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="116" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N116" s="6">
         <v>113</v>
       </c>
@@ -6470,14 +6292,14 @@
       <c r="Q116" s="6"/>
       <c r="R116" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S116" s="16">
         <f t="shared" si="7"/>
         <v>46176</v>
       </c>
     </row>
-    <row r="117" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="117" spans="14:19" x14ac:dyDescent="0.3">
       <c r="N117" s="6">
         <v>114</v>
       </c>
@@ -6491,14 +6313,14 @@
       <c r="Q117" s="6"/>
       <c r="R117" s="6">
         <f t="shared" si="8"/>
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="S117" s="16">
         <f t="shared" si="7"/>
         <v>46177</v>
       </c>
     </row>
-    <row r="118" spans="14:19" x14ac:dyDescent="0.25">
+    <row r="118" spans="14:19" x14ac:dyDescent="0.3">
       <c r="S118" s="5"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Backlog atualizado e separado por sprints
</commit_message>
<xml_diff>
--- a/Documentações/Backlog.xlsx
+++ b/Documentações/Backlog.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathe\OneDrive\Área de Trabalho\ThermoChain\Documentações\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9043B5DC-6179-4972-B9FC-F6B2F63B3114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9158A729-86B7-43D7-98AC-F1DF5A4FB052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{88668B19-0EBA-47FC-AF05-5256D7A9BC46}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{88668B19-0EBA-47FC-AF05-5256D7A9BC46}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Backlog" sheetId="1" r:id="rId1"/>
+    <sheet name="Sprint01" sheetId="2" r:id="rId2"/>
+    <sheet name="Sprint02" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="120">
   <si>
     <t>Projeto no github</t>
   </si>
@@ -860,7 +862,7 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Planilha1!$P$3:$P$117</c:f>
+              <c:f>Backlog!$P$3:$P$117</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="115"/>
@@ -1223,7 +1225,15 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Pendente</c:v>
+            <c:strRef>
+              <c:f>Backlog!$R$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>272</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:tx>
           <c:spPr>
             <a:ln w="34925" cap="rnd">
@@ -1245,10 +1255,10 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Planilha1!$R$3:$R$58</c:f>
+              <c:f>Backlog!$R$3:$R$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="56"/>
+                <c:ptCount val="60"/>
                 <c:pt idx="0">
                   <c:v>272</c:v>
                 </c:pt>
@@ -1415,6 +1425,18 @@
                   <c:v>103</c:v>
                 </c:pt>
                 <c:pt idx="55">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="59">
                   <c:v>90</c:v>
                 </c:pt>
               </c:numCache>
@@ -1515,6 +1537,7 @@
             </a:p>
           </c:txPr>
         </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2653,29 +2676,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{552007D4-E79E-4A61-AC31-FF3BEBBC1490}">
   <dimension ref="A2:T118"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.5546875" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="5" max="5" width="45.6640625" customWidth="1"/>
-    <col min="6" max="6" width="53.33203125" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" customWidth="1"/>
-    <col min="9" max="9" width="9.6640625" customWidth="1"/>
-    <col min="10" max="10" width="15.6640625" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="15.109375" customWidth="1"/>
-    <col min="13" max="13" width="8.88671875" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="45.7109375" customWidth="1"/>
+    <col min="6" max="6" width="53.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" customWidth="1"/>
+    <col min="16" max="16" width="17.7109375" customWidth="1"/>
     <col min="17" max="17" width="21" customWidth="1"/>
-    <col min="18" max="18" width="13.5546875" customWidth="1"/>
-    <col min="19" max="19" width="13.88671875" customWidth="1"/>
-    <col min="20" max="20" width="11.6640625" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" customWidth="1"/>
+    <col min="19" max="19" width="13.85546875" customWidth="1"/>
+    <col min="20" max="20" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
         <v>59</v>
       </c>
@@ -2728,7 +2751,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
         <v>63</v>
       </c>
@@ -2783,7 +2806,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>60</v>
       </c>
@@ -2841,7 +2864,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
         <v>61</v>
       </c>
@@ -2898,7 +2921,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>64</v>
       </c>
@@ -2952,7 +2975,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E7" s="19" t="s">
         <v>4</v>
       </c>
@@ -3000,7 +3023,7 @@
         <v>46067</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>101</v>
       </c>
@@ -3055,7 +3078,7 @@
         <v>46068</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>102</v>
       </c>
@@ -3109,7 +3132,7 @@
         <v>46069</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>103</v>
       </c>
@@ -3164,7 +3187,7 @@
         <v>46070</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="s">
         <v>114</v>
       </c>
@@ -3218,7 +3241,7 @@
         <v>46071</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E12" s="19" t="s">
         <v>9</v>
       </c>
@@ -3266,7 +3289,7 @@
         <v>46072</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="E13" s="19" t="s">
         <v>10</v>
@@ -3315,7 +3338,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="E14" s="19" t="s">
         <v>11</v>
@@ -3364,7 +3387,7 @@
         <v>46074</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E15" s="19" t="s">
         <v>12</v>
       </c>
@@ -3412,7 +3435,7 @@
         <v>46075</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E16" s="19" t="s">
         <v>13</v>
       </c>
@@ -3460,7 +3483,7 @@
         <v>46076</v>
       </c>
     </row>
-    <row r="17" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E17" s="19" t="s">
         <v>14</v>
       </c>
@@ -3508,7 +3531,7 @@
         <v>46077</v>
       </c>
     </row>
-    <row r="18" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E18" s="19" t="s">
         <v>15</v>
       </c>
@@ -3556,7 +3579,7 @@
         <v>46078</v>
       </c>
     </row>
-    <row r="19" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E19" s="19" t="s">
         <v>24</v>
       </c>
@@ -3604,7 +3627,7 @@
         <v>46079</v>
       </c>
     </row>
-    <row r="20" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E20" s="19" t="s">
         <v>25</v>
       </c>
@@ -3650,7 +3673,7 @@
         <v>46080</v>
       </c>
     </row>
-    <row r="21" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E21" s="19" t="s">
         <v>26</v>
       </c>
@@ -3698,7 +3721,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="22" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E22" s="19" t="s">
         <v>27</v>
       </c>
@@ -3746,7 +3769,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="23" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="23" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E23" s="19" t="s">
         <v>28</v>
       </c>
@@ -3794,7 +3817,7 @@
         <v>46083</v>
       </c>
     </row>
-    <row r="24" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="24" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E24" s="19" t="s">
         <v>29</v>
       </c>
@@ -3842,7 +3865,7 @@
         <v>46084</v>
       </c>
     </row>
-    <row r="25" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E25" s="19" t="s">
         <v>30</v>
       </c>
@@ -3888,7 +3911,7 @@
         <v>46085</v>
       </c>
     </row>
-    <row r="26" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E26" s="19" t="s">
         <v>31</v>
       </c>
@@ -3936,7 +3959,7 @@
         <v>46086</v>
       </c>
     </row>
-    <row r="27" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E27" s="19" t="s">
         <v>32</v>
       </c>
@@ -3984,7 +4007,7 @@
         <v>46087</v>
       </c>
     </row>
-    <row r="28" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E28" s="19" t="s">
         <v>33</v>
       </c>
@@ -4032,7 +4055,7 @@
         <v>46088</v>
       </c>
     </row>
-    <row r="29" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E29" s="19" t="s">
         <v>34</v>
       </c>
@@ -4080,7 +4103,7 @@
         <v>46089</v>
       </c>
     </row>
-    <row r="30" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E30" s="19" t="s">
         <v>35</v>
       </c>
@@ -4128,7 +4151,7 @@
         <v>46090</v>
       </c>
     </row>
-    <row r="31" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E31" s="19" t="s">
         <v>36</v>
       </c>
@@ -4174,7 +4197,7 @@
         <v>46091</v>
       </c>
     </row>
-    <row r="32" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="32" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E32" s="19" t="s">
         <v>37</v>
       </c>
@@ -4222,7 +4245,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="33" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E33" s="19" t="s">
         <v>38</v>
       </c>
@@ -4270,7 +4293,7 @@
         <v>46093</v>
       </c>
     </row>
-    <row r="34" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E34" s="19" t="s">
         <v>39</v>
       </c>
@@ -4316,7 +4339,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="35" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E35" s="19" t="s">
         <v>90</v>
       </c>
@@ -4362,7 +4385,7 @@
         <v>46095</v>
       </c>
     </row>
-    <row r="36" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E36" s="19" t="s">
         <v>91</v>
       </c>
@@ -4408,7 +4431,7 @@
         <v>46096</v>
       </c>
     </row>
-    <row r="37" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E37" s="19" t="s">
         <v>92</v>
       </c>
@@ -4454,7 +4477,7 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="38" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E38" s="19" t="s">
         <v>93</v>
       </c>
@@ -4500,7 +4523,7 @@
         <v>46098</v>
       </c>
     </row>
-    <row r="39" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E39" s="31" t="s">
         <v>94</v>
       </c>
@@ -4546,7 +4569,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="40" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E40" s="32" t="s">
         <v>116</v>
       </c>
@@ -4592,7 +4615,7 @@
         <v>46100</v>
       </c>
     </row>
-    <row r="41" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E41" s="39" t="s">
         <v>118</v>
       </c>
@@ -4638,7 +4661,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="42" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N42" s="6">
         <v>39</v>
       </c>
@@ -4662,7 +4685,7 @@
         <v>46102</v>
       </c>
     </row>
-    <row r="43" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N43" s="6">
         <v>40</v>
       </c>
@@ -4686,7 +4709,7 @@
         <v>46103</v>
       </c>
     </row>
-    <row r="44" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="44" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N44" s="6">
         <v>41</v>
       </c>
@@ -4710,7 +4733,7 @@
         <v>46104</v>
       </c>
     </row>
-    <row r="45" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="45" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N45" s="6">
         <v>42</v>
       </c>
@@ -4734,7 +4757,7 @@
         <v>46105</v>
       </c>
     </row>
-    <row r="46" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="46" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N46" s="6">
         <v>43</v>
       </c>
@@ -4758,7 +4781,7 @@
         <v>46106</v>
       </c>
     </row>
-    <row r="47" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="47" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N47" s="6">
         <v>44</v>
       </c>
@@ -4782,7 +4805,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="48" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="48" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N48" s="6">
         <v>45</v>
       </c>
@@ -4806,7 +4829,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="49" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="49" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N49" s="6">
         <v>46</v>
       </c>
@@ -4830,7 +4853,7 @@
         <v>46109</v>
       </c>
     </row>
-    <row r="50" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="50" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N50" s="6">
         <v>47</v>
       </c>
@@ -4854,7 +4877,7 @@
         <v>46110</v>
       </c>
     </row>
-    <row r="51" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="51" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N51" s="6">
         <v>48</v>
       </c>
@@ -4878,7 +4901,7 @@
         <v>46111</v>
       </c>
     </row>
-    <row r="52" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="52" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N52" s="6">
         <v>49</v>
       </c>
@@ -4902,7 +4925,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="53" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="53" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N53" s="6">
         <v>50</v>
       </c>
@@ -4926,7 +4949,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="54" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="54" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N54" s="6">
         <v>51</v>
       </c>
@@ -4950,7 +4973,7 @@
         <v>46114</v>
       </c>
     </row>
-    <row r="55" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="55" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N55" s="6">
         <v>52</v>
       </c>
@@ -4974,7 +4997,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="56" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="56" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N56" s="6">
         <v>53</v>
       </c>
@@ -4998,7 +5021,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="57" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="57" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N57" s="6">
         <v>54</v>
       </c>
@@ -5022,7 +5045,7 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="58" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="58" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N58" s="6">
         <v>55</v>
       </c>
@@ -5046,7 +5069,7 @@
         <v>46118</v>
       </c>
     </row>
-    <row r="59" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="59" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N59" s="6">
         <v>56</v>
       </c>
@@ -5058,7 +5081,9 @@
         <f t="shared" si="1"/>
         <v>104</v>
       </c>
-      <c r="Q59" s="6"/>
+      <c r="Q59" s="6">
+        <v>0</v>
+      </c>
       <c r="R59" s="6">
         <f t="shared" si="3"/>
         <v>90</v>
@@ -5068,7 +5093,7 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="60" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="60" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N60" s="6">
         <v>57</v>
       </c>
@@ -5080,7 +5105,9 @@
         <f t="shared" si="1"/>
         <v>101</v>
       </c>
-      <c r="Q60" s="6"/>
+      <c r="Q60" s="6">
+        <v>0</v>
+      </c>
       <c r="R60" s="6">
         <f t="shared" si="3"/>
         <v>90</v>
@@ -5090,7 +5117,7 @@
         <v>46120</v>
       </c>
     </row>
-    <row r="61" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="61" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N61" s="6">
         <v>58</v>
       </c>
@@ -5102,7 +5129,9 @@
         <f t="shared" si="1"/>
         <v>98</v>
       </c>
-      <c r="Q61" s="6"/>
+      <c r="Q61" s="6">
+        <v>0</v>
+      </c>
       <c r="R61" s="6">
         <f t="shared" si="3"/>
         <v>90</v>
@@ -5112,7 +5141,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="62" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="62" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N62" s="6">
         <v>59</v>
       </c>
@@ -5124,7 +5153,9 @@
         <f t="shared" si="1"/>
         <v>95</v>
       </c>
-      <c r="Q62" s="6"/>
+      <c r="Q62" s="6">
+        <v>0</v>
+      </c>
       <c r="R62" s="6">
         <f t="shared" si="3"/>
         <v>90</v>
@@ -5134,7 +5165,7 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="63" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="63" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N63" s="6">
         <v>60</v>
       </c>
@@ -5156,7 +5187,7 @@
         <v>46123</v>
       </c>
     </row>
-    <row r="64" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="64" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N64" s="6">
         <v>61</v>
       </c>
@@ -5178,7 +5209,7 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="65" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="65" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N65" s="6">
         <v>62</v>
       </c>
@@ -5200,7 +5231,7 @@
         <v>46125</v>
       </c>
     </row>
-    <row r="66" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="66" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N66" s="6">
         <v>63</v>
       </c>
@@ -5222,7 +5253,7 @@
         <v>46126</v>
       </c>
     </row>
-    <row r="67" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="67" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N67" s="6">
         <v>64</v>
       </c>
@@ -5244,7 +5275,7 @@
         <v>46127</v>
       </c>
     </row>
-    <row r="68" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="68" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N68" s="6">
         <v>65</v>
       </c>
@@ -5266,7 +5297,7 @@
         <v>46128</v>
       </c>
     </row>
-    <row r="69" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="69" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N69" s="6">
         <v>66</v>
       </c>
@@ -5288,7 +5319,7 @@
         <v>46129</v>
       </c>
     </row>
-    <row r="70" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="70" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N70" s="6">
         <v>67</v>
       </c>
@@ -5310,7 +5341,7 @@
         <v>46130</v>
       </c>
     </row>
-    <row r="71" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="71" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N71" s="6">
         <v>68</v>
       </c>
@@ -5332,7 +5363,7 @@
         <v>46131</v>
       </c>
     </row>
-    <row r="72" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="72" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N72" s="6">
         <v>69</v>
       </c>
@@ -5354,7 +5385,7 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="73" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="73" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N73" s="6">
         <v>70</v>
       </c>
@@ -5376,7 +5407,7 @@
         <v>46133</v>
       </c>
     </row>
-    <row r="74" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="74" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N74" s="6">
         <v>71</v>
       </c>
@@ -5398,7 +5429,7 @@
         <v>46134</v>
       </c>
     </row>
-    <row r="75" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="75" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N75" s="6">
         <v>72</v>
       </c>
@@ -5420,7 +5451,7 @@
         <v>46135</v>
       </c>
     </row>
-    <row r="76" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="76" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N76" s="6">
         <v>73</v>
       </c>
@@ -5442,7 +5473,7 @@
         <v>46136</v>
       </c>
     </row>
-    <row r="77" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="77" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N77" s="6">
         <v>74</v>
       </c>
@@ -5464,7 +5495,7 @@
         <v>46137</v>
       </c>
     </row>
-    <row r="78" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="78" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N78" s="6">
         <v>75</v>
       </c>
@@ -5486,7 +5517,7 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="79" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="79" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N79" s="6">
         <v>76</v>
       </c>
@@ -5508,7 +5539,7 @@
         <v>46139</v>
       </c>
     </row>
-    <row r="80" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="80" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N80" s="6">
         <v>77</v>
       </c>
@@ -5530,7 +5561,7 @@
         <v>46140</v>
       </c>
     </row>
-    <row r="81" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="81" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N81" s="6">
         <v>78</v>
       </c>
@@ -5552,7 +5583,7 @@
         <v>46141</v>
       </c>
     </row>
-    <row r="82" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="82" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N82" s="6">
         <v>79</v>
       </c>
@@ -5574,7 +5605,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="83" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="83" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N83" s="6">
         <v>80</v>
       </c>
@@ -5596,7 +5627,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="84" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="84" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N84" s="6">
         <v>81</v>
       </c>
@@ -5618,7 +5649,7 @@
         <v>46144</v>
       </c>
     </row>
-    <row r="85" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="85" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N85" s="6">
         <v>82</v>
       </c>
@@ -5640,7 +5671,7 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="86" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="86" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N86" s="6">
         <v>83</v>
       </c>
@@ -5662,7 +5693,7 @@
         <v>46146</v>
       </c>
     </row>
-    <row r="87" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="87" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N87" s="6">
         <v>84</v>
       </c>
@@ -5684,7 +5715,7 @@
         <v>46147</v>
       </c>
     </row>
-    <row r="88" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="88" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N88" s="6">
         <v>85</v>
       </c>
@@ -5706,7 +5737,7 @@
         <v>46148</v>
       </c>
     </row>
-    <row r="89" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="89" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N89" s="6">
         <v>86</v>
       </c>
@@ -5728,7 +5759,7 @@
         <v>46149</v>
       </c>
     </row>
-    <row r="90" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="90" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N90" s="6">
         <v>87</v>
       </c>
@@ -5750,7 +5781,7 @@
         <v>46150</v>
       </c>
     </row>
-    <row r="91" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="91" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N91" s="6">
         <v>88</v>
       </c>
@@ -5772,7 +5803,7 @@
         <v>46151</v>
       </c>
     </row>
-    <row r="92" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="92" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N92" s="6">
         <v>89</v>
       </c>
@@ -5794,7 +5825,7 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="93" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="93" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N93" s="6">
         <v>90</v>
       </c>
@@ -5816,7 +5847,7 @@
         <v>46153</v>
       </c>
     </row>
-    <row r="94" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="94" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N94" s="6">
         <v>91</v>
       </c>
@@ -5837,7 +5868,7 @@
         <v>46154</v>
       </c>
     </row>
-    <row r="95" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="95" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N95" s="6">
         <v>92</v>
       </c>
@@ -5858,7 +5889,7 @@
         <v>46155</v>
       </c>
     </row>
-    <row r="96" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="96" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N96" s="6">
         <v>93</v>
       </c>
@@ -5879,7 +5910,7 @@
         <v>46156</v>
       </c>
     </row>
-    <row r="97" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="97" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N97" s="6">
         <v>94</v>
       </c>
@@ -5900,7 +5931,7 @@
         <v>46157</v>
       </c>
     </row>
-    <row r="98" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="98" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N98" s="6">
         <v>95</v>
       </c>
@@ -5921,7 +5952,7 @@
         <v>46158</v>
       </c>
     </row>
-    <row r="99" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="99" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N99" s="6">
         <v>96</v>
       </c>
@@ -5942,7 +5973,7 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="100" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="100" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N100" s="6">
         <v>97</v>
       </c>
@@ -5963,7 +5994,7 @@
         <v>46160</v>
       </c>
     </row>
-    <row r="101" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="101" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N101" s="6">
         <v>98</v>
       </c>
@@ -5984,7 +6015,7 @@
         <v>46161</v>
       </c>
     </row>
-    <row r="102" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="102" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N102" s="6">
         <v>99</v>
       </c>
@@ -6005,7 +6036,7 @@
         <v>46162</v>
       </c>
     </row>
-    <row r="103" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="103" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N103" s="6">
         <v>100</v>
       </c>
@@ -6026,7 +6057,7 @@
         <v>46163</v>
       </c>
     </row>
-    <row r="104" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="104" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N104" s="6">
         <v>101</v>
       </c>
@@ -6047,7 +6078,7 @@
         <v>46164</v>
       </c>
     </row>
-    <row r="105" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="105" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N105" s="6">
         <v>102</v>
       </c>
@@ -6068,7 +6099,7 @@
         <v>46165</v>
       </c>
     </row>
-    <row r="106" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="106" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N106" s="6">
         <v>103</v>
       </c>
@@ -6089,7 +6120,7 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="107" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="107" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N107" s="6">
         <v>104</v>
       </c>
@@ -6110,7 +6141,7 @@
         <v>46167</v>
       </c>
     </row>
-    <row r="108" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="108" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N108" s="6">
         <v>105</v>
       </c>
@@ -6131,7 +6162,7 @@
         <v>46168</v>
       </c>
     </row>
-    <row r="109" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="109" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N109" s="6">
         <v>106</v>
       </c>
@@ -6152,7 +6183,7 @@
         <v>46169</v>
       </c>
     </row>
-    <row r="110" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="110" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N110" s="6">
         <v>107</v>
       </c>
@@ -6173,7 +6204,7 @@
         <v>46170</v>
       </c>
     </row>
-    <row r="111" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="111" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N111" s="6">
         <v>108</v>
       </c>
@@ -6194,7 +6225,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="112" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="112" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N112" s="6">
         <v>109</v>
       </c>
@@ -6215,7 +6246,7 @@
         <v>46172</v>
       </c>
     </row>
-    <row r="113" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="113" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N113" s="6">
         <v>110</v>
       </c>
@@ -6236,7 +6267,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="114" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="114" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N114" s="6">
         <v>111</v>
       </c>
@@ -6257,7 +6288,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="115" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="115" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N115" s="6">
         <v>112</v>
       </c>
@@ -6278,7 +6309,7 @@
         <v>46175</v>
       </c>
     </row>
-    <row r="116" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="116" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N116" s="6">
         <v>113</v>
       </c>
@@ -6299,7 +6330,7 @@
         <v>46176</v>
       </c>
     </row>
-    <row r="117" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="117" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N117" s="6">
         <v>114</v>
       </c>
@@ -6320,7 +6351,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="118" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="118" spans="14:19" x14ac:dyDescent="0.25">
       <c r="S118" s="5"/>
     </row>
   </sheetData>
@@ -6383,4 +6414,948 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2FF7EC3-657A-4070-AE9C-58B86EBA694A}">
+  <dimension ref="E5:O21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="35" customWidth="1"/>
+    <col min="6" max="6" width="55.28515625" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="5:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E6" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" s="23">
+        <v>3</v>
+      </c>
+      <c r="J6" s="21">
+        <v>3</v>
+      </c>
+      <c r="K6" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="N6" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="O6" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E7" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" s="25">
+        <v>8</v>
+      </c>
+      <c r="J7" s="20">
+        <v>1</v>
+      </c>
+      <c r="K7" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="N7" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="O7" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E8" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="27">
+        <v>13</v>
+      </c>
+      <c r="J8" s="20">
+        <v>1</v>
+      </c>
+      <c r="K8" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="N8" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="O8" s="4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E9" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="27">
+        <v>13</v>
+      </c>
+      <c r="J9" s="20">
+        <v>1</v>
+      </c>
+      <c r="K9" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="N9" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="O9" s="4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E10" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H10" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="I10" s="27">
+        <v>13</v>
+      </c>
+      <c r="J10" s="22">
+        <v>2</v>
+      </c>
+      <c r="K10" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E11" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" s="25">
+        <v>8</v>
+      </c>
+      <c r="J11" s="20">
+        <v>1</v>
+      </c>
+      <c r="K11" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E12" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="24">
+        <v>5</v>
+      </c>
+      <c r="J12" s="22">
+        <v>2</v>
+      </c>
+      <c r="K12" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E13" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I13" s="23">
+        <v>3</v>
+      </c>
+      <c r="J13" s="21">
+        <v>3</v>
+      </c>
+      <c r="K13" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E14" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H14" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" s="27">
+        <v>13</v>
+      </c>
+      <c r="J14" s="20">
+        <v>1</v>
+      </c>
+      <c r="K14" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E15" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H15" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="I15" s="25">
+        <v>8</v>
+      </c>
+      <c r="J15" s="20">
+        <v>1</v>
+      </c>
+      <c r="K15" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E16" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I16" s="24">
+        <v>5</v>
+      </c>
+      <c r="J16" s="22">
+        <v>2</v>
+      </c>
+      <c r="K16" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E17" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="G17" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I17" s="24">
+        <v>5</v>
+      </c>
+      <c r="J17" s="22">
+        <v>2</v>
+      </c>
+      <c r="K17" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E18" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="G18" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I18" s="23">
+        <v>3</v>
+      </c>
+      <c r="J18" s="21">
+        <v>3</v>
+      </c>
+      <c r="K18" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E19" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I19" s="24">
+        <v>5</v>
+      </c>
+      <c r="J19" s="21">
+        <v>3</v>
+      </c>
+      <c r="K19" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E20" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H20" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I20" s="23">
+        <v>3</v>
+      </c>
+      <c r="J20" s="20">
+        <v>1</v>
+      </c>
+      <c r="K20" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E21" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H21" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I21" s="24">
+        <v>5</v>
+      </c>
+      <c r="J21" s="20">
+        <v>1</v>
+      </c>
+      <c r="K21" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E0C898B-4D90-40D3-AB4B-229545D6799D}">
+  <dimension ref="E5:O20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="46.28515625" customWidth="1"/>
+    <col min="6" max="6" width="53.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E5" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" s="23">
+        <v>3</v>
+      </c>
+      <c r="J5" s="22">
+        <v>2</v>
+      </c>
+      <c r="K5" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="N5" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E6" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" s="23">
+        <v>3</v>
+      </c>
+      <c r="J6" s="22">
+        <v>2</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L6" s="4"/>
+      <c r="N6" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="O6" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E7" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="H7" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" s="25">
+        <v>8</v>
+      </c>
+      <c r="J7" s="21">
+        <v>3</v>
+      </c>
+      <c r="K7" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="N7" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="O7" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E8" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="27">
+        <v>13</v>
+      </c>
+      <c r="J8" s="20">
+        <v>1</v>
+      </c>
+      <c r="K8" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="N8" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="O8" s="4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E9" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="27">
+        <v>13</v>
+      </c>
+      <c r="J9" s="20">
+        <v>1</v>
+      </c>
+      <c r="K9" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="N9" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="O9" s="4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E10" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="I10" s="25">
+        <v>8</v>
+      </c>
+      <c r="J10" s="22">
+        <v>2</v>
+      </c>
+      <c r="K10" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E11" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" s="25">
+        <v>8</v>
+      </c>
+      <c r="J11" s="22">
+        <v>2</v>
+      </c>
+      <c r="K11" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L11" s="4"/>
+    </row>
+    <row r="12" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E12" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I12" s="23">
+        <v>3</v>
+      </c>
+      <c r="J12" s="21">
+        <v>3</v>
+      </c>
+      <c r="K12" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E13" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I13" s="24">
+        <v>5</v>
+      </c>
+      <c r="J13" s="21">
+        <v>3</v>
+      </c>
+      <c r="K13" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E14" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="H14" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="I14" s="25">
+        <v>8</v>
+      </c>
+      <c r="J14" s="20">
+        <v>1</v>
+      </c>
+      <c r="K14" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E15" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="H15" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="I15" s="25">
+        <v>8</v>
+      </c>
+      <c r="J15" s="22">
+        <v>2</v>
+      </c>
+      <c r="K15" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="5:15" x14ac:dyDescent="0.25">
+      <c r="E16" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I16" s="24">
+        <v>5</v>
+      </c>
+      <c r="J16" s="20">
+        <v>1</v>
+      </c>
+      <c r="K16" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E17" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I17" s="24">
+        <v>5</v>
+      </c>
+      <c r="J17" s="20">
+        <v>1</v>
+      </c>
+      <c r="K17" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L17" s="4"/>
+    </row>
+    <row r="18" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E18" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H18" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="I18" s="24">
+        <v>5</v>
+      </c>
+      <c r="J18" s="21">
+        <v>3</v>
+      </c>
+      <c r="K18" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E19" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G19" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="H19" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I19" s="23">
+        <v>3</v>
+      </c>
+      <c r="J19" s="21">
+        <v>3</v>
+      </c>
+      <c r="K19" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E20" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G20" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="H20" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="I20" s="23">
+        <v>3</v>
+      </c>
+      <c r="J20" s="20">
+        <v>1</v>
+      </c>
+      <c r="K20" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L20" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: refatorando responsáveis no backlog
</commit_message>
<xml_diff>
--- a/Documentações/Backlog.xlsx
+++ b/Documentações/Backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathe\OneDrive\Área de Trabalho\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\albuq\Repositorios\ThermoChain\Documentações\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{60A16035-DD5B-47F5-925C-A529310C7E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2550136C-158B-40BF-921F-D0CEC0D08F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{88668B19-0EBA-47FC-AF05-5256D7A9BC46}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{88668B19-0EBA-47FC-AF05-5256D7A9BC46}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -2683,29 +2683,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{552007D4-E79E-4A61-AC31-FF3BEBBC1490}">
   <dimension ref="A2:T118"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.5546875" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="5" max="5" width="45.6640625" customWidth="1"/>
-    <col min="6" max="6" width="53.33203125" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" customWidth="1"/>
-    <col min="9" max="9" width="9.6640625" customWidth="1"/>
-    <col min="10" max="10" width="15.6640625" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="15.109375" customWidth="1"/>
-    <col min="13" max="13" width="8.88671875" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="45.7109375" customWidth="1"/>
+    <col min="6" max="6" width="53.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" customWidth="1"/>
+    <col min="16" max="16" width="17.7109375" customWidth="1"/>
     <col min="17" max="17" width="21" customWidth="1"/>
-    <col min="18" max="18" width="13.5546875" customWidth="1"/>
-    <col min="19" max="19" width="13.88671875" customWidth="1"/>
-    <col min="20" max="20" width="11.6640625" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" customWidth="1"/>
+    <col min="19" max="19" width="13.85546875" customWidth="1"/>
+    <col min="20" max="20" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
         <v>59</v>
       </c>
@@ -2758,7 +2758,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
         <v>63</v>
       </c>
@@ -2813,7 +2813,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>60</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
         <v>61</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>64</v>
       </c>
@@ -2982,7 +2982,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E7" s="19" t="s">
         <v>4</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>46067</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>101</v>
       </c>
@@ -3085,7 +3085,7 @@
         <v>46068</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>102</v>
       </c>
@@ -3139,7 +3139,7 @@
         <v>46069</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>103</v>
       </c>
@@ -3194,7 +3194,7 @@
         <v>46070</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="s">
         <v>114</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>46071</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E12" s="19" t="s">
         <v>9</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>46072</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="E13" s="19" t="s">
         <v>10</v>
@@ -3345,7 +3345,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="E14" s="19" t="s">
         <v>11</v>
@@ -3394,7 +3394,7 @@
         <v>46074</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E15" s="19" t="s">
         <v>12</v>
       </c>
@@ -3442,7 +3442,7 @@
         <v>46075</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E16" s="19" t="s">
         <v>13</v>
       </c>
@@ -3490,7 +3490,7 @@
         <v>46076</v>
       </c>
     </row>
-    <row r="17" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E17" s="19" t="s">
         <v>14</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>46077</v>
       </c>
     </row>
-    <row r="18" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E18" s="19" t="s">
         <v>15</v>
       </c>
@@ -3586,7 +3586,7 @@
         <v>46078</v>
       </c>
     </row>
-    <row r="19" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E19" s="19" t="s">
         <v>24</v>
       </c>
@@ -3634,7 +3634,7 @@
         <v>46079</v>
       </c>
     </row>
-    <row r="20" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E20" s="19" t="s">
         <v>25</v>
       </c>
@@ -3682,7 +3682,7 @@
         <v>46080</v>
       </c>
     </row>
-    <row r="21" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E21" s="19" t="s">
         <v>26</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="22" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E22" s="19" t="s">
         <v>27</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="23" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="23" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E23" s="19" t="s">
         <v>28</v>
       </c>
@@ -3826,7 +3826,7 @@
         <v>46083</v>
       </c>
     </row>
-    <row r="24" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="24" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E24" s="19" t="s">
         <v>29</v>
       </c>
@@ -3874,7 +3874,7 @@
         <v>46084</v>
       </c>
     </row>
-    <row r="25" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E25" s="19" t="s">
         <v>30</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>46085</v>
       </c>
     </row>
-    <row r="26" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E26" s="19" t="s">
         <v>31</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>46086</v>
       </c>
     </row>
-    <row r="27" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E27" s="19" t="s">
         <v>32</v>
       </c>
@@ -4018,7 +4018,7 @@
         <v>46087</v>
       </c>
     </row>
-    <row r="28" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E28" s="19" t="s">
         <v>33</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>46088</v>
       </c>
     </row>
-    <row r="29" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E29" s="19" t="s">
         <v>34</v>
       </c>
@@ -4114,7 +4114,7 @@
         <v>46089</v>
       </c>
     </row>
-    <row r="30" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E30" s="19" t="s">
         <v>35</v>
       </c>
@@ -4162,7 +4162,7 @@
         <v>46090</v>
       </c>
     </row>
-    <row r="31" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E31" s="19" t="s">
         <v>36</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>46091</v>
       </c>
     </row>
-    <row r="32" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="32" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E32" s="19" t="s">
         <v>37</v>
       </c>
@@ -4258,7 +4258,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="33" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E33" s="19" t="s">
         <v>38</v>
       </c>
@@ -4306,7 +4306,7 @@
         <v>46093</v>
       </c>
     </row>
-    <row r="34" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E34" s="19" t="s">
         <v>39</v>
       </c>
@@ -4329,7 +4329,7 @@
         <v>88</v>
       </c>
       <c r="L34" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="N34" s="6">
         <v>31</v>
@@ -4354,7 +4354,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="35" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E35" s="19" t="s">
         <v>90</v>
       </c>
@@ -4400,7 +4400,7 @@
         <v>46095</v>
       </c>
     </row>
-    <row r="36" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E36" s="19" t="s">
         <v>91</v>
       </c>
@@ -4446,7 +4446,7 @@
         <v>46096</v>
       </c>
     </row>
-    <row r="37" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E37" s="19" t="s">
         <v>92</v>
       </c>
@@ -4492,7 +4492,7 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="38" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E38" s="19" t="s">
         <v>93</v>
       </c>
@@ -4538,7 +4538,7 @@
         <v>46098</v>
       </c>
     </row>
-    <row r="39" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E39" s="31" t="s">
         <v>94</v>
       </c>
@@ -4584,7 +4584,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="40" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E40" s="32" t="s">
         <v>116</v>
       </c>
@@ -4630,7 +4630,7 @@
         <v>46100</v>
       </c>
     </row>
-    <row r="41" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="5:19" x14ac:dyDescent="0.25">
       <c r="E41" s="39" t="s">
         <v>118</v>
       </c>
@@ -4676,7 +4676,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="42" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N42" s="6">
         <v>39</v>
       </c>
@@ -4700,7 +4700,7 @@
         <v>46102</v>
       </c>
     </row>
-    <row r="43" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N43" s="6">
         <v>40</v>
       </c>
@@ -4724,7 +4724,7 @@
         <v>46103</v>
       </c>
     </row>
-    <row r="44" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="44" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N44" s="6">
         <v>41</v>
       </c>
@@ -4748,7 +4748,7 @@
         <v>46104</v>
       </c>
     </row>
-    <row r="45" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="45" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N45" s="6">
         <v>42</v>
       </c>
@@ -4772,7 +4772,7 @@
         <v>46105</v>
       </c>
     </row>
-    <row r="46" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="46" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N46" s="6">
         <v>43</v>
       </c>
@@ -4796,7 +4796,7 @@
         <v>46106</v>
       </c>
     </row>
-    <row r="47" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="47" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N47" s="6">
         <v>44</v>
       </c>
@@ -4820,7 +4820,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="48" spans="5:19" x14ac:dyDescent="0.3">
+    <row r="48" spans="5:19" x14ac:dyDescent="0.25">
       <c r="N48" s="6">
         <v>45</v>
       </c>
@@ -4844,7 +4844,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="49" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="49" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N49" s="6">
         <v>46</v>
       </c>
@@ -4868,7 +4868,7 @@
         <v>46109</v>
       </c>
     </row>
-    <row r="50" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="50" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N50" s="6">
         <v>47</v>
       </c>
@@ -4892,7 +4892,7 @@
         <v>46110</v>
       </c>
     </row>
-    <row r="51" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="51" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N51" s="6">
         <v>48</v>
       </c>
@@ -4916,7 +4916,7 @@
         <v>46111</v>
       </c>
     </row>
-    <row r="52" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="52" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N52" s="6">
         <v>49</v>
       </c>
@@ -4940,7 +4940,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="53" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="53" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N53" s="6">
         <v>50</v>
       </c>
@@ -4964,7 +4964,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="54" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="54" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N54" s="6">
         <v>51</v>
       </c>
@@ -4988,7 +4988,7 @@
         <v>46114</v>
       </c>
     </row>
-    <row r="55" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="55" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N55" s="6">
         <v>52</v>
       </c>
@@ -5012,7 +5012,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="56" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="56" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N56" s="6">
         <v>53</v>
       </c>
@@ -5036,7 +5036,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="57" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="57" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N57" s="6">
         <v>54</v>
       </c>
@@ -5060,7 +5060,7 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="58" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="58" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N58" s="6">
         <v>55</v>
       </c>
@@ -5084,7 +5084,7 @@
         <v>46118</v>
       </c>
     </row>
-    <row r="59" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="59" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N59" s="6">
         <v>56</v>
       </c>
@@ -5108,7 +5108,7 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="60" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="60" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N60" s="6">
         <v>57</v>
       </c>
@@ -5132,7 +5132,7 @@
         <v>46120</v>
       </c>
     </row>
-    <row r="61" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="61" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N61" s="6">
         <v>58</v>
       </c>
@@ -5156,7 +5156,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="62" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="62" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N62" s="6">
         <v>59</v>
       </c>
@@ -5180,7 +5180,7 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="63" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="63" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N63" s="6">
         <v>60</v>
       </c>
@@ -5204,7 +5204,7 @@
         <v>46123</v>
       </c>
     </row>
-    <row r="64" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="64" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N64" s="6">
         <v>61</v>
       </c>
@@ -5228,7 +5228,7 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="65" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="65" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N65" s="6">
         <v>62</v>
       </c>
@@ -5250,7 +5250,7 @@
         <v>46125</v>
       </c>
     </row>
-    <row r="66" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="66" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N66" s="6">
         <v>63</v>
       </c>
@@ -5272,7 +5272,7 @@
         <v>46126</v>
       </c>
     </row>
-    <row r="67" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="67" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N67" s="6">
         <v>64</v>
       </c>
@@ -5294,7 +5294,7 @@
         <v>46127</v>
       </c>
     </row>
-    <row r="68" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="68" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N68" s="6">
         <v>65</v>
       </c>
@@ -5316,7 +5316,7 @@
         <v>46128</v>
       </c>
     </row>
-    <row r="69" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="69" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N69" s="6">
         <v>66</v>
       </c>
@@ -5338,7 +5338,7 @@
         <v>46129</v>
       </c>
     </row>
-    <row r="70" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="70" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N70" s="6">
         <v>67</v>
       </c>
@@ -5360,7 +5360,7 @@
         <v>46130</v>
       </c>
     </row>
-    <row r="71" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="71" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N71" s="6">
         <v>68</v>
       </c>
@@ -5382,7 +5382,7 @@
         <v>46131</v>
       </c>
     </row>
-    <row r="72" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="72" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N72" s="6">
         <v>69</v>
       </c>
@@ -5404,7 +5404,7 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="73" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="73" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N73" s="6">
         <v>70</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>46133</v>
       </c>
     </row>
-    <row r="74" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="74" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N74" s="6">
         <v>71</v>
       </c>
@@ -5448,7 +5448,7 @@
         <v>46134</v>
       </c>
     </row>
-    <row r="75" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="75" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N75" s="6">
         <v>72</v>
       </c>
@@ -5470,7 +5470,7 @@
         <v>46135</v>
       </c>
     </row>
-    <row r="76" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="76" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N76" s="6">
         <v>73</v>
       </c>
@@ -5492,7 +5492,7 @@
         <v>46136</v>
       </c>
     </row>
-    <row r="77" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="77" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N77" s="6">
         <v>74</v>
       </c>
@@ -5514,7 +5514,7 @@
         <v>46137</v>
       </c>
     </row>
-    <row r="78" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="78" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N78" s="6">
         <v>75</v>
       </c>
@@ -5536,7 +5536,7 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="79" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="79" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N79" s="6">
         <v>76</v>
       </c>
@@ -5558,7 +5558,7 @@
         <v>46139</v>
       </c>
     </row>
-    <row r="80" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="80" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N80" s="6">
         <v>77</v>
       </c>
@@ -5580,7 +5580,7 @@
         <v>46140</v>
       </c>
     </row>
-    <row r="81" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="81" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N81" s="6">
         <v>78</v>
       </c>
@@ -5602,7 +5602,7 @@
         <v>46141</v>
       </c>
     </row>
-    <row r="82" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="82" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N82" s="6">
         <v>79</v>
       </c>
@@ -5624,7 +5624,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="83" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="83" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N83" s="6">
         <v>80</v>
       </c>
@@ -5646,7 +5646,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="84" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="84" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N84" s="6">
         <v>81</v>
       </c>
@@ -5668,7 +5668,7 @@
         <v>46144</v>
       </c>
     </row>
-    <row r="85" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="85" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N85" s="6">
         <v>82</v>
       </c>
@@ -5690,7 +5690,7 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="86" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="86" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N86" s="6">
         <v>83</v>
       </c>
@@ -5712,7 +5712,7 @@
         <v>46146</v>
       </c>
     </row>
-    <row r="87" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="87" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N87" s="6">
         <v>84</v>
       </c>
@@ -5734,7 +5734,7 @@
         <v>46147</v>
       </c>
     </row>
-    <row r="88" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="88" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N88" s="6">
         <v>85</v>
       </c>
@@ -5756,7 +5756,7 @@
         <v>46148</v>
       </c>
     </row>
-    <row r="89" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="89" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N89" s="6">
         <v>86</v>
       </c>
@@ -5778,7 +5778,7 @@
         <v>46149</v>
       </c>
     </row>
-    <row r="90" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="90" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N90" s="6">
         <v>87</v>
       </c>
@@ -5800,7 +5800,7 @@
         <v>46150</v>
       </c>
     </row>
-    <row r="91" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="91" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N91" s="6">
         <v>88</v>
       </c>
@@ -5822,7 +5822,7 @@
         <v>46151</v>
       </c>
     </row>
-    <row r="92" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="92" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N92" s="6">
         <v>89</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="93" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="93" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N93" s="6">
         <v>90</v>
       </c>
@@ -5866,7 +5866,7 @@
         <v>46153</v>
       </c>
     </row>
-    <row r="94" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="94" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N94" s="6">
         <v>91</v>
       </c>
@@ -5887,7 +5887,7 @@
         <v>46154</v>
       </c>
     </row>
-    <row r="95" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="95" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N95" s="6">
         <v>92</v>
       </c>
@@ -5908,7 +5908,7 @@
         <v>46155</v>
       </c>
     </row>
-    <row r="96" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="96" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N96" s="6">
         <v>93</v>
       </c>
@@ -5929,7 +5929,7 @@
         <v>46156</v>
       </c>
     </row>
-    <row r="97" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="97" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N97" s="6">
         <v>94</v>
       </c>
@@ -5950,7 +5950,7 @@
         <v>46157</v>
       </c>
     </row>
-    <row r="98" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="98" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N98" s="6">
         <v>95</v>
       </c>
@@ -5971,7 +5971,7 @@
         <v>46158</v>
       </c>
     </row>
-    <row r="99" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="99" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N99" s="6">
         <v>96</v>
       </c>
@@ -5992,7 +5992,7 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="100" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="100" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N100" s="6">
         <v>97</v>
       </c>
@@ -6013,7 +6013,7 @@
         <v>46160</v>
       </c>
     </row>
-    <row r="101" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="101" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N101" s="6">
         <v>98</v>
       </c>
@@ -6034,7 +6034,7 @@
         <v>46161</v>
       </c>
     </row>
-    <row r="102" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="102" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N102" s="6">
         <v>99</v>
       </c>
@@ -6055,7 +6055,7 @@
         <v>46162</v>
       </c>
     </row>
-    <row r="103" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="103" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N103" s="6">
         <v>100</v>
       </c>
@@ -6076,7 +6076,7 @@
         <v>46163</v>
       </c>
     </row>
-    <row r="104" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="104" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N104" s="6">
         <v>101</v>
       </c>
@@ -6097,7 +6097,7 @@
         <v>46164</v>
       </c>
     </row>
-    <row r="105" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="105" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N105" s="6">
         <v>102</v>
       </c>
@@ -6118,7 +6118,7 @@
         <v>46165</v>
       </c>
     </row>
-    <row r="106" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="106" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N106" s="6">
         <v>103</v>
       </c>
@@ -6139,7 +6139,7 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="107" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="107" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N107" s="6">
         <v>104</v>
       </c>
@@ -6160,7 +6160,7 @@
         <v>46167</v>
       </c>
     </row>
-    <row r="108" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="108" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N108" s="6">
         <v>105</v>
       </c>
@@ -6181,7 +6181,7 @@
         <v>46168</v>
       </c>
     </row>
-    <row r="109" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="109" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N109" s="6">
         <v>106</v>
       </c>
@@ -6202,7 +6202,7 @@
         <v>46169</v>
       </c>
     </row>
-    <row r="110" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="110" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N110" s="6">
         <v>107</v>
       </c>
@@ -6223,7 +6223,7 @@
         <v>46170</v>
       </c>
     </row>
-    <row r="111" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="111" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N111" s="6">
         <v>108</v>
       </c>
@@ -6244,7 +6244,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="112" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="112" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N112" s="6">
         <v>109</v>
       </c>
@@ -6265,7 +6265,7 @@
         <v>46172</v>
       </c>
     </row>
-    <row r="113" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="113" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N113" s="6">
         <v>110</v>
       </c>
@@ -6286,7 +6286,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="114" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="114" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N114" s="6">
         <v>111</v>
       </c>
@@ -6307,7 +6307,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="115" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="115" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N115" s="6">
         <v>112</v>
       </c>
@@ -6328,7 +6328,7 @@
         <v>46175</v>
       </c>
     </row>
-    <row r="116" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="116" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N116" s="6">
         <v>113</v>
       </c>
@@ -6349,7 +6349,7 @@
         <v>46176</v>
       </c>
     </row>
-    <row r="117" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="117" spans="14:19" x14ac:dyDescent="0.25">
       <c r="N117" s="6">
         <v>114</v>
       </c>
@@ -6370,7 +6370,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="118" spans="14:19" x14ac:dyDescent="0.3">
+    <row r="118" spans="14:19" x14ac:dyDescent="0.25">
       <c r="S118" s="5"/>
     </row>
   </sheetData>

</xml_diff>